<commit_message>
新测试 	modified:   0 zombie type/sun/sun_config.json 	modified:   0 zombie type/sun/sun_info.xlsx
</commit_message>
<xml_diff>
--- a/0 zombie type/sun/sun_info.xlsx
+++ b/0 zombie type/sun/sun_info.xlsx
@@ -7,7 +7,8 @@
     <workbookView windowHeight="16660"/>
   </bookViews>
   <sheets>
-    <sheet name="main" sheetId="5" r:id="rId1"/>
+    <sheet name="NE1" sheetId="6" r:id="rId1"/>
+    <sheet name="N6E1.5 68" sheetId="5" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="34">
   <si>
     <t>地图类型</t>
   </si>
@@ -68,64 +69,67 @@
     <t>用户ID</t>
   </si>
   <si>
+    <t>白眼</t>
+  </si>
+  <si>
+    <t>模式ID</t>
+  </si>
+  <si>
+    <t>密度</t>
+  </si>
+  <si>
+    <t>已完成f数（偶数）</t>
+  </si>
+  <si>
+    <t>冲关选卡数</t>
+  </si>
+  <si>
+    <t>舞王</t>
+  </si>
+  <si>
+    <t>阳光初值</t>
+  </si>
+  <si>
+    <t>破阵阳光值</t>
+  </si>
+  <si>
+    <t>阳光无上限</t>
+  </si>
+  <si>
+    <t>否</t>
+  </si>
+  <si>
+    <t>计算模式</t>
+  </si>
+  <si>
+    <t>1-随机种子模拟</t>
+  </si>
+  <si>
+    <t>模式1</t>
+  </si>
+  <si>
+    <t>模拟次数</t>
+  </si>
+  <si>
+    <t>输出种子数</t>
+  </si>
+  <si>
+    <t>模式2</t>
+  </si>
+  <si>
+    <t>种子</t>
+  </si>
+  <si>
+    <t>6A25E7B6</t>
+  </si>
+  <si>
     <t>气球</t>
   </si>
   <si>
-    <t>模式ID</t>
-  </si>
-  <si>
-    <t>舞王</t>
-  </si>
-  <si>
-    <t>已完成f数（偶数）</t>
-  </si>
-  <si>
-    <t>白眼</t>
-  </si>
-  <si>
-    <t>冲关选卡数</t>
-  </si>
-  <si>
     <t>撑杆</t>
   </si>
   <si>
-    <t>阳光初值</t>
-  </si>
-  <si>
-    <t>密度</t>
-  </si>
-  <si>
-    <t>破阵阳光值</t>
-  </si>
-  <si>
-    <t>阳光无上限</t>
-  </si>
-  <si>
     <t>是</t>
-  </si>
-  <si>
-    <t>计算模式</t>
-  </si>
-  <si>
-    <t>1-随机种子模拟</t>
-  </si>
-  <si>
-    <t>模式1</t>
-  </si>
-  <si>
-    <t>模拟次数</t>
-  </si>
-  <si>
-    <t>输出种子数</t>
-  </si>
-  <si>
-    <t>模式2</t>
-  </si>
-  <si>
-    <t>种子</t>
-  </si>
-  <si>
-    <t>6A25E7B6</t>
   </si>
 </sst>
 </file>
@@ -1278,6 +1282,334 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr defaultColWidth="9.16346153846154" defaultRowHeight="16.8" outlineLevelCol="5"/>
+  <cols>
+    <col min="1" max="1" width="29.6923076923077" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.1538461538462" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.16346153846154" style="1"/>
+    <col min="4" max="5" width="7" style="1" customWidth="1"/>
+    <col min="6" max="6" width="9.69230769230769" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.16346153846154" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" spans="1:6">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" s="1" customFormat="1" spans="4:6">
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" s="1" customFormat="1" spans="1:6">
+      <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="3">
+        <v>43.8763</v>
+      </c>
+    </row>
+    <row r="4" s="1" customFormat="1" spans="1:6">
+      <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="3">
+        <v>10000</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="3">
+        <v>-295.3125</v>
+      </c>
+    </row>
+    <row r="5" s="1" customFormat="1" spans="4:6">
+      <c r="D5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="3">
+        <v>-359.375</v>
+      </c>
+    </row>
+    <row r="6" s="1" customFormat="1" spans="1:6">
+      <c r="A6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="3">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="3">
+        <v>54.6875</v>
+      </c>
+    </row>
+    <row r="7" s="1" customFormat="1" spans="1:6">
+      <c r="A7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="3">
+        <v>13</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="3">
+        <v>-76.5625</v>
+      </c>
+    </row>
+    <row r="8" s="1" customFormat="1" spans="1:6">
+      <c r="A8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="3">
+        <v>2000</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="3">
+        <v>-50</v>
+      </c>
+    </row>
+    <row r="9" s="1" customFormat="1" spans="1:6">
+      <c r="A9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="3">
+        <v>5000</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="3">
+        <v>-76.5625</v>
+      </c>
+    </row>
+    <row r="10" s="1" customFormat="1" spans="1:6">
+      <c r="A10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="3">
+        <v>10000</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="3">
+        <v>-56.25</v>
+      </c>
+    </row>
+    <row r="11" s="1" customFormat="1" spans="1:6">
+      <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="3">
+        <v>-500</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="3">
+        <v>-50</v>
+      </c>
+    </row>
+    <row r="12" s="1" customFormat="1" spans="1:6">
+      <c r="A12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" s="1" customFormat="1" spans="4:6">
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" s="1" customFormat="1" spans="1:6">
+      <c r="A14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" s="1" customFormat="1" spans="4:6">
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" s="1" customFormat="1" spans="1:6">
+      <c r="A16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" s="1" customFormat="1" spans="1:6">
+      <c r="A17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="3">
+        <v>10000</v>
+      </c>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+    </row>
+    <row r="18" s="1" customFormat="1" spans="1:6">
+      <c r="A18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="3">
+        <v>10</v>
+      </c>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+    </row>
+    <row r="19" s="1" customFormat="1" spans="4:6">
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+    </row>
+    <row r="20" s="1" customFormat="1" spans="1:6">
+      <c r="A20" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+    </row>
+    <row r="21" s="1" customFormat="1" spans="1:6">
+      <c r="A21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+    </row>
+    <row r="22" s="1" customFormat="1" spans="1:6">
+      <c r="A22"/>
+      <c r="B22"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+    </row>
+    <row r="23" s="1" customFormat="1" spans="1:6">
+      <c r="A23"/>
+      <c r="B23"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+    </row>
+    <row r="24" s="1" customFormat="1" spans="1:6">
+      <c r="A24"/>
+      <c r="B24"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+    </row>
+    <row r="25" s="1" customFormat="1" spans="4:6">
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A20:B20"/>
+  </mergeCells>
+  <dataValidations count="6">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1 A4:B4 A6 B17 B21 B6:B10 F3:F25"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1">
+      <formula1>"DE/MGE/AQE,NE,PE/FE,RE/ME"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3">
+      <formula1>"1/-1,1/0"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11 D9:D11 E9:E10 D12:E25 D3:E8">
+      <formula1>"空,路障,撑杆,铁桶,读报,铁门,橄榄,舞王,潜水,冰车,海豚,小丑,气球,矿工,跳跳,蹦极,扶梯,投篮,白眼,红眼,密度"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B12">
+      <formula1>"否,是"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B14">
+      <formula1>"1-随机种子模拟,2-固定种子模拟"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:F25"/>
   <sheetFormatPr defaultColWidth="9.16346153846154" defaultRowHeight="16.8" outlineLevelCol="5"/>
@@ -1367,7 +1699,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>8</v>
@@ -1384,7 +1716,7 @@
         <v>13</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>8</v>
@@ -1401,7 +1733,7 @@
         <v>2000</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>8</v>
@@ -1412,13 +1744,13 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B9" s="3">
         <v>500000</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>8</v>
@@ -1429,13 +1761,13 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3">
         <v>10000</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>8</v>
@@ -1446,7 +1778,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3">
         <v>-500</v>
@@ -1455,7 +1787,7 @@
         <v>11</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F11" s="3">
         <v>60.15625</v>
@@ -1463,16 +1795,16 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="F12" s="3">
         <v>-52.34375</v>
@@ -1485,10 +1817,10 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
@@ -1501,7 +1833,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B16" s="2"/>
       <c r="D16" s="3"/>
@@ -1510,7 +1842,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B17" s="3">
         <v>100</v>
@@ -1521,7 +1853,7 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B18" s="3">
         <v>10</v>
@@ -1537,7 +1869,7 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B20" s="2"/>
       <c r="D20" s="3"/>
@@ -1546,10 +1878,10 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
@@ -1588,15 +1920,12 @@
     <mergeCell ref="A20:B20"/>
   </mergeCells>
   <dataValidations count="6">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1 F3 A4 B4 F4 A6 B6 B7 B8 B9 B10 B17 B21 F5:F25"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1 A4:B4 A6 B17 B21 B6:B10 F3:F25"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1">
       <formula1>"DE/MGE/AQE,NE,PE/FE,RE/ME"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3">
       <formula1>"1/-1,1/0"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3 D4 D5:D25 E3:E10 E11:E25">
-      <formula1>"空,路障,撑杆,铁桶,读报,铁门,橄榄,舞王,潜水,冰车,海豚,小丑,气球,矿工,跳跳,蹦极,扶梯,投篮,白眼,红眼,密度"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B12">
       <formula1>"否,是"</formula1>
@@ -1604,6 +1933,9 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B14">
       <formula1>"1-随机种子模拟,2-固定种子模拟"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:E25">
+      <formula1>"空,路障,撑杆,铁桶,读报,铁门,橄榄,舞王,潜水,冰车,海豚,小丑,气球,矿工,跳跳,蹦极,扶梯,投篮,白眼,红眼,密度"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>